<commit_message>
TEST: reduced peak 556 damage
</commit_message>
<xml_diff>
--- a/changes/556-barrels.xlsx
+++ b/changes/556-barrels.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yifan/Documents/deadline-balancing/changes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F619A4B-317D-AE46-AB42-20C3B248B9B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A146A695-CBF3-4E32-87BF-B206C8A11765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="760" windowWidth="38640" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="m4-barrels" sheetId="1" r:id="rId1"/>
@@ -122,21 +122,12 @@
     <t>base</t>
   </si>
   <si>
-    <t>fn_scar_l_254mm_barrel</t>
-  </si>
-  <si>
     <t>FN SCAR-L 254mm</t>
   </si>
   <si>
-    <t>fn_scar_l_355mm_barrel</t>
-  </si>
-  <si>
     <t>FN SCAR-L 355mm</t>
   </si>
   <si>
-    <t>fn_scar_l_457mm_barrel</t>
-  </si>
-  <si>
     <t>FN SCAR-L 457mm</t>
   </si>
   <si>
@@ -300,6 +291,15 @@
   </si>
   <si>
     <t>new weight</t>
+  </si>
+  <si>
+    <t>aft_mk_16_457mm_barrel</t>
+  </si>
+  <si>
+    <t>aft_mk_16_355mm_barrel</t>
+  </si>
+  <si>
+    <t>aft_mk_16_254mm_barrel</t>
   </si>
 </sst>
 </file>
@@ -1149,19 +1149,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.33203125" customWidth="1"/>
-    <col min="2" max="2" width="27.1640625" customWidth="1"/>
-    <col min="3" max="25" width="6.6640625" customWidth="1"/>
+    <col min="1" max="1" width="29.42578125" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" customWidth="1"/>
+    <col min="3" max="25" width="6.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1184,7 +1184,7 @@
         <v>8</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I2" t="s">
         <v>9</v>
@@ -1193,7 +1193,7 @@
         <v>10</v>
       </c>
       <c r="K2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="L2" t="s">
         <v>11</v>
@@ -1214,22 +1214,22 @@
         <v>14</v>
       </c>
       <c r="S2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="T2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="U2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="V2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="X2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1252,7 +1252,7 @@
         <v>-0.32</v>
       </c>
       <c r="I3">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="J3">
         <v>262</v>
@@ -1264,8 +1264,8 @@
         <v>5000</v>
       </c>
       <c r="N3">
-        <f>C3-D3*20-E3*0.8-F3*0.6-H3*5+I3*10+J3/300</f>
-        <v>-2.5266666666666655</v>
+        <f>C3-D3*20-E3*0.8-F3*0.6-H3*5+I3*15+J3/300</f>
+        <v>-2.0266666666666655</v>
       </c>
       <c r="P3">
         <v>0.18</v>
@@ -1288,8 +1288,8 @@
         <v>0.98799999999999999</v>
       </c>
       <c r="V3">
-        <f>0+(Q3-14.5)*-0.045</f>
-        <v>-0.42749999999999999</v>
+        <f>0+(Q3-14.5)*-0.043</f>
+        <v>-0.40849999999999997</v>
       </c>
       <c r="X3">
         <v>349.95</v>
@@ -1299,9 +1299,9 @@
         <v>2099.6999999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
@@ -1322,7 +1322,7 @@
         <v>-0.24</v>
       </c>
       <c r="I4">
-        <v>0.26</v>
+        <v>0.21</v>
       </c>
       <c r="J4">
         <v>179</v>
@@ -1334,8 +1334,8 @@
         <v>1600</v>
       </c>
       <c r="N4">
-        <f t="shared" ref="N4:N39" si="0">C4-D4*20-E4*0.8-F4*0.6-H4*5+I4*10+J4/300</f>
-        <v>-7.4033333333333351</v>
+        <f t="shared" ref="N4:N39" si="0">C4-D4*20-E4*0.8-F4*0.6-H4*5+I4*15+J4/300</f>
+        <v>-6.8533333333333344</v>
       </c>
       <c r="P4">
         <v>0.18</v>
@@ -1355,8 +1355,8 @@
         <v>0.84000000000000008</v>
       </c>
       <c r="V4">
-        <f t="shared" ref="V4:V34" si="3">0+(Q4-14.5)*-0.045</f>
-        <v>-0.2475</v>
+        <f t="shared" ref="V4:V38" si="3">0+(Q4-14.5)*-0.043</f>
+        <v>-0.23649999999999999</v>
       </c>
       <c r="X4">
         <v>344.99</v>
@@ -1370,9 +1370,9 @@
         <v>0.80681818181818177</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B5" t="s">
         <v>18</v>
@@ -1384,16 +1384,16 @@
         <v>0.94</v>
       </c>
       <c r="E5">
-        <v>-11</v>
+        <v>-12</v>
       </c>
       <c r="F5">
         <v>-12</v>
       </c>
       <c r="H5">
-        <v>-0.26</v>
+        <v>-0.22</v>
       </c>
       <c r="I5">
-        <v>0.26</v>
+        <v>0.21</v>
       </c>
       <c r="J5">
         <v>191</v>
@@ -1406,7 +1406,7 @@
       </c>
       <c r="N5">
         <f t="shared" si="0"/>
-        <v>-8.2633333333333301</v>
+        <v>-7.1133333333333297</v>
       </c>
       <c r="P5">
         <v>0.18</v>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="V5">
         <f t="shared" si="3"/>
-        <v>-0.2475</v>
+        <v>-0.23649999999999999</v>
       </c>
       <c r="X5">
         <v>349.99</v>
@@ -1440,9 +1440,9 @@
         <v>2099.94</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B6" t="s">
         <v>19</v>
@@ -1460,10 +1460,10 @@
         <v>-9</v>
       </c>
       <c r="H6">
-        <v>-0.15</v>
+        <v>-0.13</v>
       </c>
       <c r="I6">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="J6">
         <v>131</v>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="N6">
         <f t="shared" si="0"/>
-        <v>-6.0133333333333345</v>
+        <v>-5.4633333333333338</v>
       </c>
       <c r="P6">
         <v>0.15</v>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="V6">
         <f t="shared" si="3"/>
-        <v>-0.1575</v>
+        <v>-0.15049999999999999</v>
       </c>
       <c r="X6">
         <v>372</v>
@@ -1510,9 +1510,9 @@
         <v>2232</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B7" t="s">
         <v>20</v>
@@ -1533,7 +1533,7 @@
         <v>-0.05</v>
       </c>
       <c r="I7">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="J7">
         <v>108</v>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="N7">
         <f t="shared" si="0"/>
-        <v>-6.1899999999999995</v>
+        <v>-5.9899999999999993</v>
       </c>
       <c r="P7">
         <v>0.15</v>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="V7">
         <f t="shared" si="3"/>
-        <v>-6.7500000000000004E-2</v>
+        <v>-6.4500000000000002E-2</v>
       </c>
       <c r="X7">
         <v>329.99</v>
@@ -1577,9 +1577,9 @@
         <v>1979.94</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B8" t="s">
         <v>21</v>
@@ -1600,7 +1600,7 @@
         <v>-7.0000000000000007E-2</v>
       </c>
       <c r="I8">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="J8">
         <v>78</v>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="N8">
         <f t="shared" si="0"/>
-        <v>-6.9899999999999993</v>
+        <v>-6.6899999999999995</v>
       </c>
       <c r="P8">
         <v>0.12</v>
@@ -1634,7 +1634,7 @@
       </c>
       <c r="V8">
         <f t="shared" si="3"/>
-        <v>-6.7500000000000004E-2</v>
+        <v>-6.4500000000000002E-2</v>
       </c>
       <c r="X8">
         <v>279.99</v>
@@ -1644,12 +1644,12 @@
         <v>1679.94</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C9">
         <v>-1</v>
@@ -1677,7 +1677,7 @@
       </c>
       <c r="N9">
         <f t="shared" si="0"/>
-        <v>-6.35</v>
+        <v>-6.15</v>
       </c>
       <c r="P9">
         <v>0.12</v>
@@ -1711,12 +1711,12 @@
         <v>2094</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B10" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="N10">
         <f t="shared" si="0"/>
-        <v>-6.2899999999999991</v>
+        <v>-6.1899999999999995</v>
       </c>
       <c r="P10">
         <v>0.12</v>
@@ -1772,9 +1772,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B11" t="s">
         <v>27</v>
@@ -1786,16 +1786,16 @@
         <v>0.61</v>
       </c>
       <c r="E11">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="F11">
         <v>-4</v>
       </c>
       <c r="H11">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="I11">
-        <v>-0.01</v>
+        <v>0.01</v>
       </c>
       <c r="J11">
         <v>37</v>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="N11">
         <f t="shared" si="0"/>
-        <v>-4.9266666666666659</v>
+        <v>-5.5266666666666664</v>
       </c>
       <c r="P11">
         <v>0.15</v>
@@ -1832,15 +1832,15 @@
       </c>
       <c r="V11">
         <f t="shared" si="3"/>
-        <v>3.6000000000000032E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.2">
+        <v>3.4400000000000028E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -1858,7 +1858,7 @@
         <v>0.09</v>
       </c>
       <c r="I12">
-        <v>-0.04</v>
+        <v>-0.02</v>
       </c>
       <c r="J12">
         <v>-34</v>
@@ -1868,7 +1868,7 @@
       </c>
       <c r="N12">
         <f t="shared" si="0"/>
-        <v>-6.5633333333333344</v>
+        <v>-6.4633333333333338</v>
       </c>
       <c r="P12">
         <v>0.12</v>
@@ -1889,7 +1889,7 @@
       </c>
       <c r="V12">
         <f t="shared" si="3"/>
-        <v>0.09</v>
+        <v>8.5999999999999993E-2</v>
       </c>
       <c r="X12">
         <v>338</v>
@@ -1899,9 +1899,9 @@
         <v>2028</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B13" t="s">
         <v>25</v>
@@ -1922,7 +1922,7 @@
         <v>0.13</v>
       </c>
       <c r="I13">
-        <v>-7.0000000000000007E-2</v>
+        <v>-0.05</v>
       </c>
       <c r="J13">
         <v>-72</v>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="N13">
         <f t="shared" si="0"/>
-        <v>-6.1900000000000013</v>
+        <v>-6.2400000000000011</v>
       </c>
       <c r="P13">
         <v>0.12</v>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="V13">
         <f t="shared" si="3"/>
-        <v>0.13500000000000001</v>
+        <v>0.129</v>
       </c>
       <c r="X13">
         <v>155</v>
@@ -1963,12 +1963,12 @@
         <v>930</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B14" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C14">
         <v>3</v>
@@ -1983,10 +1983,10 @@
         <v>-1</v>
       </c>
       <c r="H14">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="I14">
-        <v>-0.1</v>
+        <v>-0.08</v>
       </c>
       <c r="J14">
         <v>-113</v>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="N14">
         <f t="shared" si="0"/>
-        <v>-6.4766666666666666</v>
+        <v>-6.626666666666666</v>
       </c>
       <c r="P14">
         <v>0.12</v>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="V14">
         <f t="shared" si="3"/>
-        <v>0.18</v>
+        <v>0.17199999999999999</v>
       </c>
       <c r="X14">
         <v>299</v>
@@ -2027,12 +2027,12 @@
         <v>1794</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B15" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C15">
         <v>4</v>
@@ -2050,7 +2050,7 @@
         <v>0.3</v>
       </c>
       <c r="I15">
-        <v>-0.15</v>
+        <v>-0.13</v>
       </c>
       <c r="J15">
         <v>-266</v>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="N15">
         <f t="shared" si="0"/>
-        <v>-6.0866666666666669</v>
+        <v>-6.5366666666666671</v>
       </c>
       <c r="P15">
         <v>0.09</v>
@@ -2084,16 +2084,16 @@
       </c>
       <c r="V15">
         <f t="shared" si="3"/>
-        <v>0.315</v>
+        <v>0.30099999999999999</v>
       </c>
       <c r="Y15">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B16" t="s">
         <v>22</v>
@@ -2114,7 +2114,7 @@
         <v>0.4</v>
       </c>
       <c r="I16">
-        <v>-0.2</v>
+        <v>-0.18</v>
       </c>
       <c r="J16">
         <v>-450</v>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="N16">
         <f t="shared" si="0"/>
-        <v>-5.9</v>
+        <v>-6.6</v>
       </c>
       <c r="P16">
         <v>7.0000000000000007E-2</v>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="V16">
         <f t="shared" si="3"/>
-        <v>0.42749999999999999</v>
+        <v>0.40849999999999997</v>
       </c>
       <c r="X16">
         <v>149.94999999999999</v>
@@ -2158,7 +2158,7 @@
         <v>899.69999999999993</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="N17">
         <f t="shared" si="0"/>
-        <v>-35.286666666666662</v>
+        <v>-37.286666666666662</v>
       </c>
       <c r="P17">
         <v>0.05</v>
@@ -2218,14 +2218,14 @@
       </c>
       <c r="V17">
         <f t="shared" si="3"/>
-        <v>0.5625</v>
+        <v>0.53749999999999998</v>
       </c>
       <c r="Y17">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="N18">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2236,15 +2236,15 @@
       </c>
       <c r="V18">
         <f t="shared" si="3"/>
-        <v>0.65249999999999997</v>
-      </c>
-    </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.2">
+        <v>0.62349999999999994</v>
+      </c>
+    </row>
+    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B19" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C19">
         <v>4</v>
@@ -2259,10 +2259,10 @@
         <v>3</v>
       </c>
       <c r="H19">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="I19">
-        <v>-0.12</v>
+        <v>-0.11</v>
       </c>
       <c r="J19">
         <v>-140</v>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="N19">
         <f t="shared" si="0"/>
-        <v>-11.116666666666665</v>
+        <v>-11.516666666666666</v>
       </c>
       <c r="P19">
         <v>0.04</v>
@@ -2293,15 +2293,15 @@
       </c>
       <c r="V19">
         <f t="shared" si="3"/>
-        <v>0.2475</v>
-      </c>
-    </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.2">
+        <v>0.23649999999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C20">
         <v>3</v>
@@ -2319,7 +2319,7 @@
         <v>0.18</v>
       </c>
       <c r="I20">
-        <v>-0.09</v>
+        <v>-0.08</v>
       </c>
       <c r="J20">
         <v>-100</v>
@@ -2329,7 +2329,7 @@
       </c>
       <c r="N20">
         <f t="shared" si="0"/>
-        <v>-11.133333333333335</v>
+        <v>-11.433333333333334</v>
       </c>
       <c r="P20">
         <v>0.04</v>
@@ -2341,7 +2341,7 @@
         <v>0.02</v>
       </c>
       <c r="S20">
-        <f>ROUND(Q20*0.033+P49+R20, 2)</f>
+        <f t="shared" ref="S20:S28" si="5">ROUND(Q20*0.033+P49+R20, 2)</f>
         <v>0.36</v>
       </c>
       <c r="U20">
@@ -2350,15 +2350,15 @@
       </c>
       <c r="V20">
         <f t="shared" si="3"/>
-        <v>0.18449999999999997</v>
-      </c>
-    </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.2">
+        <v>0.17629999999999996</v>
+      </c>
+    </row>
+    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C21">
         <v>2</v>
@@ -2376,7 +2376,7 @@
         <v>0.15</v>
       </c>
       <c r="I21">
-        <v>-7.0000000000000007E-2</v>
+        <v>-0.06</v>
       </c>
       <c r="J21">
         <v>-80</v>
@@ -2386,7 +2386,7 @@
       </c>
       <c r="N21">
         <f t="shared" si="0"/>
-        <v>-10.516666666666666</v>
+        <v>-10.716666666666667</v>
       </c>
       <c r="P21">
         <v>0.04</v>
@@ -2398,7 +2398,7 @@
         <v>0</v>
       </c>
       <c r="S21">
-        <f>ROUND(Q21*0.033+P50+R21, 2)</f>
+        <f t="shared" si="5"/>
         <v>0.36</v>
       </c>
       <c r="U21">
@@ -2407,15 +2407,15 @@
       </c>
       <c r="V21">
         <f t="shared" si="3"/>
-        <v>0.1575</v>
-      </c>
-    </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.2">
+        <v>0.15049999999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B22" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -2433,7 +2433,7 @@
         <v>0.08</v>
       </c>
       <c r="I22">
-        <v>-0.03</v>
+        <v>-0.02</v>
       </c>
       <c r="J22">
         <v>-30</v>
@@ -2455,7 +2455,7 @@
         <v>0</v>
       </c>
       <c r="S22">
-        <f>ROUND(Q22*0.033+P51+R22, 2)</f>
+        <f t="shared" si="5"/>
         <v>0.41</v>
       </c>
       <c r="U22">
@@ -2464,15 +2464,15 @@
       </c>
       <c r="V22">
         <f t="shared" si="3"/>
-        <v>0.09</v>
-      </c>
-    </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.2">
+        <v>8.5999999999999993E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -2500,7 +2500,7 @@
       </c>
       <c r="N23">
         <f t="shared" si="0"/>
-        <v>-12.533333333333333</v>
+        <v>-12.383333333333335</v>
       </c>
       <c r="P23">
         <v>0.04</v>
@@ -2512,7 +2512,7 @@
         <v>0.05</v>
       </c>
       <c r="S23">
-        <f>ROUND(Q23*0.033+P52+R23, 2)</f>
+        <f t="shared" si="5"/>
         <v>0.53</v>
       </c>
       <c r="U23">
@@ -2524,12 +2524,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B24" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -2557,7 +2557,7 @@
       </c>
       <c r="N24">
         <f t="shared" si="0"/>
-        <v>-11.833333333333334</v>
+        <v>-11.683333333333335</v>
       </c>
       <c r="P24">
         <v>0.04</v>
@@ -2569,7 +2569,7 @@
         <v>0.02</v>
       </c>
       <c r="S24">
-        <f>ROUND(Q24*0.033+P53+R24, 2)</f>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="U24">
@@ -2581,12 +2581,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B25" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C25">
         <v>-3</v>
@@ -2604,7 +2604,7 @@
         <v>-0.08</v>
       </c>
       <c r="I25">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="J25">
         <v>100</v>
@@ -2614,7 +2614,7 @@
       </c>
       <c r="N25">
         <f t="shared" si="0"/>
-        <v>-12.766666666666666</v>
+        <v>-12.366666666666665</v>
       </c>
       <c r="P25">
         <v>0.04</v>
@@ -2626,7 +2626,7 @@
         <v>0.05</v>
       </c>
       <c r="S25">
-        <f>ROUND(Q25*0.033+P54+R25, 2)</f>
+        <f t="shared" si="5"/>
         <v>0.59</v>
       </c>
       <c r="U25">
@@ -2635,15 +2635,15 @@
       </c>
       <c r="V25">
         <f t="shared" si="3"/>
-        <v>-0.09</v>
-      </c>
-    </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.2">
+        <v>-8.5999999999999993E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B26" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C26">
         <v>-3</v>
@@ -2661,7 +2661,7 @@
         <v>-0.1</v>
       </c>
       <c r="I26">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="J26">
         <v>100</v>
@@ -2671,7 +2671,7 @@
       </c>
       <c r="N26">
         <f t="shared" si="0"/>
-        <v>-12.066666666666665</v>
+        <v>-11.666666666666664</v>
       </c>
       <c r="P26">
         <v>0.04</v>
@@ -2683,7 +2683,7 @@
         <v>0.02</v>
       </c>
       <c r="S26">
-        <f>ROUND(Q26*0.033+P55+R26, 2)</f>
+        <f t="shared" si="5"/>
         <v>0.56000000000000005</v>
       </c>
       <c r="U26">
@@ -2692,15 +2692,15 @@
       </c>
       <c r="V26">
         <f t="shared" si="3"/>
-        <v>-0.09</v>
-      </c>
-    </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.2">
+        <v>-8.5999999999999993E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B27" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C27">
         <v>-7</v>
@@ -2715,10 +2715,10 @@
         <v>-5</v>
       </c>
       <c r="H27">
-        <v>-0.24</v>
+        <v>-0.22</v>
       </c>
       <c r="I27">
-        <v>0.25</v>
+        <v>0.21</v>
       </c>
       <c r="J27">
         <v>190</v>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="N27">
         <f t="shared" si="0"/>
-        <v>-12.666666666666668</v>
+        <v>-12.116666666666667</v>
       </c>
       <c r="P27">
         <v>0.04</v>
@@ -2740,7 +2740,7 @@
         <v>0.05</v>
       </c>
       <c r="S27">
-        <f>ROUND(Q27*0.033+P56+R27, 2)</f>
+        <f t="shared" si="5"/>
         <v>0.71</v>
       </c>
       <c r="U27">
@@ -2749,15 +2749,15 @@
       </c>
       <c r="V27">
         <f t="shared" si="3"/>
-        <v>-0.2475</v>
-      </c>
-    </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.2">
+        <v>-0.23649999999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B28" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C28">
         <v>-7</v>
@@ -2772,10 +2772,10 @@
         <v>-5</v>
       </c>
       <c r="H28">
-        <v>-0.26</v>
+        <v>-0.24</v>
       </c>
       <c r="I28">
-        <v>0.25</v>
+        <v>0.21</v>
       </c>
       <c r="J28">
         <v>190</v>
@@ -2785,7 +2785,7 @@
       </c>
       <c r="N28">
         <f t="shared" si="0"/>
-        <v>-11.966666666666665</v>
+        <v>-11.416666666666666</v>
       </c>
       <c r="P28">
         <v>0.04</v>
@@ -2797,7 +2797,7 @@
         <v>0.02</v>
       </c>
       <c r="S28">
-        <f>ROUND(Q28*0.033+P57+R28, 2)</f>
+        <f t="shared" si="5"/>
         <v>0.68</v>
       </c>
       <c r="U28">
@@ -2806,10 +2806,10 @@
       </c>
       <c r="V28">
         <f t="shared" si="3"/>
-        <v>-0.2475</v>
-      </c>
-    </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.2">
+        <v>-0.23649999999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -2828,24 +2828,24 @@
         <v>0</v>
       </c>
       <c r="S29">
-        <f>ROUND(Q29*0.033+P29+R29, 2)</f>
+        <f t="shared" ref="S29:S34" si="6">ROUND(Q29*0.033+P29+R29, 2)</f>
         <v>0</v>
       </c>
       <c r="U29">
-        <f>0.06+0.037*Q29+T29+R29</f>
+        <f t="shared" ref="U29:U34" si="7">0.06+0.037*Q29+T29+R29</f>
         <v>0.06</v>
       </c>
       <c r="V29">
         <f t="shared" si="3"/>
-        <v>0.65249999999999997</v>
-      </c>
-    </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.2">
+        <v>0.62349999999999994</v>
+      </c>
+    </row>
+    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C30" s="1">
         <v>-10</v>
@@ -2864,7 +2864,7 @@
         <v>0.1</v>
       </c>
       <c r="I30" s="1">
-        <v>0.28000000000000003</v>
+        <v>0.21</v>
       </c>
       <c r="J30" s="1">
         <v>269</v>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="N30">
         <f t="shared" si="0"/>
-        <v>-15.803333333333329</v>
+        <v>-15.453333333333331</v>
       </c>
       <c r="P30">
         <v>0.1</v>
@@ -2888,24 +2888,24 @@
         <v>0.1</v>
       </c>
       <c r="S30">
-        <f>ROUND(Q30*0.033+P30+R30, 2)</f>
+        <f t="shared" si="6"/>
         <v>1.01</v>
       </c>
       <c r="U30">
-        <f>0.06+0.037*Q30+T30+R30</f>
+        <f t="shared" si="7"/>
         <v>1.0631478000000001</v>
       </c>
       <c r="V30">
         <f t="shared" si="3"/>
-        <v>-0.44592300000000007</v>
-      </c>
-    </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.2">
+        <v>-0.42610420000000004</v>
+      </c>
+    </row>
+    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C31" s="1">
         <v>-4</v>
@@ -2924,7 +2924,7 @@
         <v>-0.24</v>
       </c>
       <c r="I31" s="1">
-        <v>0.24</v>
+        <v>0.21</v>
       </c>
       <c r="J31" s="1">
         <v>179</v>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="N31">
         <f t="shared" si="0"/>
-        <v>-8.8033333333333346</v>
+        <v>-8.0533333333333346</v>
       </c>
       <c r="P31">
         <v>0.1</v>
@@ -2945,24 +2945,24 @@
         <v>20</v>
       </c>
       <c r="S31">
-        <f>ROUND(Q31*0.033+P31+R31, 2)</f>
+        <f t="shared" si="6"/>
         <v>0.76</v>
       </c>
       <c r="U31">
-        <f>0.06+0.037*Q31+T31+R31</f>
+        <f t="shared" si="7"/>
         <v>0.8</v>
       </c>
       <c r="V31">
         <f t="shared" si="3"/>
-        <v>-0.2475</v>
-      </c>
-    </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.2">
+        <v>-0.23649999999999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C32" s="1">
         <v>-2</v>
@@ -2981,7 +2981,7 @@
         <v>-0.15</v>
       </c>
       <c r="I32" s="1">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="J32" s="1">
         <v>131</v>
@@ -2992,8 +2992,8 @@
         <v>750</v>
       </c>
       <c r="N32">
-        <f t="shared" ref="N32:N33" si="5">C32-D32*20-E32*0.8-F32*0.6-H32*5+I32*10+J32/300</f>
-        <v>-9.4133333333333322</v>
+        <f t="shared" si="0"/>
+        <v>-8.7633333333333319</v>
       </c>
       <c r="P32">
         <v>0.1</v>
@@ -3002,24 +3002,24 @@
         <v>17.992100000000001</v>
       </c>
       <c r="S32">
-        <f>ROUND(Q32*0.033+P32+R32, 2)</f>
+        <f t="shared" si="6"/>
         <v>0.69</v>
       </c>
       <c r="U32">
-        <f>0.06+0.037*Q32+T32+R32</f>
+        <f t="shared" si="7"/>
         <v>0.72570770000000007</v>
       </c>
       <c r="V32">
         <f t="shared" si="3"/>
-        <v>-0.15714450000000002</v>
-      </c>
-    </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
+        <v>-0.15016030000000002</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C33" s="1">
         <v>0</v>
@@ -3049,8 +3049,8 @@
         <v>0</v>
       </c>
       <c r="N33">
-        <f t="shared" si="5"/>
-        <v>-10.036666666666665</v>
+        <f t="shared" si="0"/>
+        <v>-9.5366666666666653</v>
       </c>
       <c r="P33">
         <v>0.1</v>
@@ -3059,24 +3059,24 @@
         <v>16.023599999999998</v>
       </c>
       <c r="S33">
-        <f>ROUND(Q33*0.033+P33+R33, 2)</f>
+        <f t="shared" si="6"/>
         <v>0.63</v>
       </c>
       <c r="U33">
-        <f>0.06+0.037*Q33+T33+R33</f>
+        <f t="shared" si="7"/>
         <v>0.65287319999999993</v>
       </c>
       <c r="V33">
         <f t="shared" si="3"/>
-        <v>-6.8561999999999915E-2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
+        <v>-6.5514799999999915E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C34" s="1">
         <v>2</v>
@@ -3095,7 +3095,7 @@
         <v>0.03</v>
       </c>
       <c r="I34" s="1">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="J34" s="1">
         <v>10</v>
@@ -3106,8 +3106,8 @@
         <v>600</v>
       </c>
       <c r="N34">
-        <f>C34-D34*20-E34*0.8-F34*0.6-H34*5+I34*10+J34/300</f>
-        <v>-9.5166666666666657</v>
+        <f t="shared" si="0"/>
+        <v>-9.3666666666666654</v>
       </c>
       <c r="P34">
         <v>0.1</v>
@@ -3116,19 +3116,19 @@
         <v>13.779500000000001</v>
       </c>
       <c r="S34">
-        <f>ROUND(Q34*0.033+P34+R34, 2)</f>
+        <f t="shared" si="6"/>
         <v>0.55000000000000004</v>
       </c>
       <c r="U34">
-        <f>0.06+0.037*Q34+T34+R34</f>
+        <f t="shared" si="7"/>
         <v>0.56984149999999989</v>
       </c>
       <c r="V34">
         <f t="shared" si="3"/>
-        <v>3.2422499999999972E-2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
+        <v>3.0981499999999974E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -3147,20 +3147,24 @@
         <v>0</v>
       </c>
       <c r="S35">
-        <f t="shared" ref="S35:S39" si="6">ROUND(Q35*0.033+P35+R35, 2)</f>
+        <f t="shared" ref="S35:S39" si="8">ROUND(Q35*0.033+P35+R35, 2)</f>
         <v>0</v>
       </c>
       <c r="U35">
         <f t="shared" si="2"/>
         <v>0.06</v>
       </c>
-    </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="V35">
+        <f t="shared" si="3"/>
+        <v>0.62349999999999994</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>33</v>
+        <v>86</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C36" s="1">
         <v>-5</v>
@@ -3169,17 +3173,17 @@
         <v>0.73</v>
       </c>
       <c r="E36" s="1">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="F36" s="1">
         <v>-4</v>
       </c>
       <c r="G36" s="1"/>
       <c r="H36" s="1">
-        <v>-0.1</v>
+        <v>-0.15</v>
       </c>
       <c r="I36" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="J36" s="1">
         <v>131</v>
@@ -3190,8 +3194,8 @@
         <v>1500</v>
       </c>
       <c r="N36">
-        <f>C36-D36*20-E36*0.8-F36*0.6-H36*5+I36*10+J36/300</f>
-        <v>-12.463333333333335</v>
+        <f t="shared" si="0"/>
+        <v>-10.413333333333334</v>
       </c>
       <c r="P36">
         <v>0.14000000000000001</v>
@@ -3207,13 +3211,17 @@
         <f t="shared" si="2"/>
         <v>0.72570770000000007</v>
       </c>
-    </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="V36">
+        <f t="shared" si="3"/>
+        <v>-0.15016030000000002</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C37" s="1">
         <v>0</v>
@@ -3229,10 +3237,10 @@
       </c>
       <c r="G37" s="1"/>
       <c r="H37" s="1">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="I37" s="1">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="J37" s="1">
         <v>17</v>
@@ -3240,11 +3248,11 @@
       <c r="K37" s="1"/>
       <c r="L37" s="1"/>
       <c r="M37" s="1">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="N37">
-        <f>C37-D37*20-E37*0.8-F37*0.6-H37*5+I37*10+J37/300</f>
-        <v>-11.943333333333333</v>
+        <f t="shared" si="0"/>
+        <v>-11.743333333333332</v>
       </c>
       <c r="P37">
         <v>0.14000000000000001</v>
@@ -3260,13 +3268,17 @@
         <f t="shared" si="2"/>
         <v>0.57712680000000005</v>
       </c>
-    </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="V37">
+        <f t="shared" si="3"/>
+        <v>2.2514800000000001E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="C38" s="1">
         <v>2</v>
@@ -3278,7 +3290,7 @@
         <v>1</v>
       </c>
       <c r="F38" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1">
@@ -3297,7 +3309,7 @@
       </c>
       <c r="N38">
         <f t="shared" si="0"/>
-        <v>-11.649999999999999</v>
+        <v>-11.449999999999998</v>
       </c>
       <c r="P38">
         <v>0.14000000000000001</v>
@@ -3306,15 +3318,19 @@
         <v>10</v>
       </c>
       <c r="S38">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.47</v>
       </c>
       <c r="U38">
         <f t="shared" si="2"/>
         <v>0.43</v>
       </c>
-    </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="V38">
+        <f t="shared" si="3"/>
+        <v>0.19349999999999998</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -3333,11 +3349,11 @@
         <v>0</v>
       </c>
       <c r="S39">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -3352,7 +3368,7 @@
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -3367,7 +3383,7 @@
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -3382,7 +3398,7 @@
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -3397,7 +3413,7 @@
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -3412,7 +3428,7 @@
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -3427,7 +3443,7 @@
       <c r="L45" s="1"/>
       <c r="M45" s="1"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>

</xml_diff>

<commit_message>
add hbar bipod and adjust harrison stats
</commit_message>
<xml_diff>
--- a/changes/556-barrels.xlsx
+++ b/changes/556-barrels.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A146A695-CBF3-4E32-87BF-B206C8A11765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F0AF886-BBE1-4276-9778-1E32E7452A1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,34 +44,43 @@
     <t>pretty_name</t>
   </si>
   <si>
+    <t>ergonomics</t>
+  </si>
+  <si>
+    <t>weight</t>
+  </si>
+  <si>
+    <t>horizontal_recoil</t>
+  </si>
+  <si>
+    <t>vertical_recoil</t>
+  </si>
+  <si>
+    <t>magazine_capacity</t>
+  </si>
+  <si>
+    <t>barrel_deviation</t>
+  </si>
+  <si>
+    <t>bullet_damage</t>
+  </si>
+  <si>
+    <t>bullet_velocity</t>
+  </si>
+  <si>
+    <t>buck_barrel_deviation</t>
+  </si>
+  <si>
+    <t>fire_rate</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
     <t>strength</t>
   </si>
   <si>
-    <t>ergonomics</t>
-  </si>
-  <si>
-    <t>weight</t>
-  </si>
-  <si>
-    <t>horizontal_recoil</t>
-  </si>
-  <si>
-    <t>vertical_recoil</t>
-  </si>
-  <si>
-    <t>magazine_capacity</t>
-  </si>
-  <si>
-    <t>bullet_damage</t>
-  </si>
-  <si>
-    <t>bullet_velocity</t>
-  </si>
-  <si>
-    <t>fire_rate</t>
-  </si>
-  <si>
-    <t>price</t>
+    <t>base</t>
   </si>
   <si>
     <t>length</t>
@@ -80,363 +89,227 @@
     <t>mod</t>
   </si>
   <si>
+    <t>old weight</t>
+  </si>
+  <si>
+    <t>gas</t>
+  </si>
+  <si>
+    <t>new weight</t>
+  </si>
+  <si>
+    <t>dev</t>
+  </si>
+  <si>
+    <t>irl price</t>
+  </si>
+  <si>
     <t>cmmg_ar_15_5.56x45_610mm_fluted_r_barrel</t>
   </si>
   <si>
-    <t>CMMG 24" Fluted AR-15 Rifle Length Gastube 5.56x45</t>
-  </si>
-  <si>
-    <t>Brownells A1 Government 20" Rifle Length Gastube 5.56x45</t>
-  </si>
-  <si>
-    <t>Brownells HBAR 20" Rifle Length Gastube 5.56x45</t>
-  </si>
-  <si>
-    <t>X-Caliber Custom 18" Spiral 6 Groove Mid Length Gastube .223 Wylde</t>
-  </si>
-  <si>
-    <t>Brownells Government 16" Mid Length Gastube 5.56x45</t>
-  </si>
-  <si>
-    <t>Brownells Socom 16" Carbine Length Gastube 5.56x45</t>
-  </si>
-  <si>
-    <t>Vertiforce Tactical AR15 5in 5.56 Nitride Barrel Custom Gastube</t>
+    <t>CmmG 24" Fluted AR-15 Rifle Length Gastube 5.56x45</t>
+  </si>
+  <si>
+    <t>whtnls_a1_m4a1_5.56x45_508mm_govt_r_barrel</t>
+  </si>
+  <si>
+    <t>Whitnalls A1 Government 20" Rifle Length Gastube 5.56x45</t>
+  </si>
+  <si>
+    <t>whtnls_m4a1_5.56x45_508mm_hbar_r_barrel</t>
+  </si>
+  <si>
+    <t>Whitnalls HBAR 20" Rifle Length Gastube 5.56x45</t>
+  </si>
+  <si>
+    <t>ex_call_ar_15_.223wylde_457mm_spiral_6groove_m_barrel</t>
+  </si>
+  <si>
+    <t>Ex-Call Custom 18" Spiral 6 Groove Mid Length Gastube .223 Wylde</t>
+  </si>
+  <si>
+    <t>whtnls_m4a1_5.56x45_406mm_govt_m_barrel</t>
+  </si>
+  <si>
+    <t>Whitnalls Government 16" Mid Length Gastube 5.56x45</t>
+  </si>
+  <si>
+    <t>whtnls_m4a1_5.56x45_406mm_socom_c_barrel</t>
+  </si>
+  <si>
+    <t>Whitnalls Socom 16" Carbine Length Gastube 5.56x45</t>
+  </si>
+  <si>
+    <t>hart_m4a1_5.56x45_368mm_socom_c_barrel</t>
+  </si>
+  <si>
+    <t>Hart Socom 14.5" Carbine Length Gastube 5.56x45</t>
+  </si>
+  <si>
+    <t>hart_m4a1_5.56x45_368mm_govt_c_barrel</t>
+  </si>
+  <si>
+    <t>Hart Government 14.5" Carbine Length Gastube 5.56x45</t>
+  </si>
+  <si>
+    <t>pac_ks1_5.56x45_348mm_heavy_dimpled_m_barrel</t>
+  </si>
+  <si>
+    <t>PAC KS-1 (L403A1) Heavy Dimpled 13.7" Mid Length Gastube 5.56x45</t>
+  </si>
+  <si>
+    <t>hart_m4a1_5.56x45_317mm_govt_c_barrel</t>
+  </si>
+  <si>
+    <t>Hart Government 12.5" Carbine Length Gastube 5.56x45</t>
+  </si>
+  <si>
+    <t>primabarrels_ar15_modern_series_5.56x45_292mm_govt_c_barrel</t>
+  </si>
+  <si>
+    <t>PrimaBarrels Modern Series Government 11.5" Carbine Length Gastube 5.56x45</t>
+  </si>
+  <si>
+    <t>hart_m4a1_5.56x45_267mm_govt_c_barrel</t>
+  </si>
+  <si>
+    <t>Hart Government 10.5" Carbine Length Gastube 5.56x45</t>
+  </si>
+  <si>
+    <t>hart_m4a1_5.56x45_190mm_govt_p_barrel</t>
+  </si>
+  <si>
+    <t>Hart Government 7.5" Pistol Length Gastube 5.56x45</t>
+  </si>
+  <si>
+    <t>quix_tacticals_ar15_127mm_5.56_nitride_barrel_custom_gastube</t>
+  </si>
+  <si>
+    <t>Quix Tacticals AR-15 Nitride 5" Custom Length Gastube 5.56x45</t>
   </si>
   <si>
     <t>custom_2inch_ar15_barrel</t>
   </si>
   <si>
-    <t>Custom 2in AR15 Barrel</t>
-  </si>
-  <si>
-    <t>Ballistic Advantage Modern Series Government 11.5" Carbine Length Gastube 5.56x45</t>
-  </si>
-  <si>
-    <t>irl price</t>
-  </si>
-  <si>
-    <t>KAC KS-1 (L403A1) Heavy Dimpled 13.7" Mid Length Gastube 5.56x45</t>
-  </si>
-  <si>
-    <t>base</t>
-  </si>
-  <si>
-    <t>FN SCAR-L 254mm</t>
-  </si>
-  <si>
-    <t>FN SCAR-L 355mm</t>
-  </si>
-  <si>
-    <t>FN SCAR-L 457mm</t>
+    <t>Custom 2" AR-15 5.56x45</t>
+  </si>
+  <si>
+    <t>kf_416c_9.0i_barrel</t>
+  </si>
+  <si>
+    <t>KF416C 9.0"</t>
+  </si>
+  <si>
+    <t>kf_416d_10.4i_barrel</t>
+  </si>
+  <si>
+    <t>KF416D 10.4"</t>
+  </si>
+  <si>
+    <t>kf_416a5_11i_barrel</t>
+  </si>
+  <si>
+    <t>KF416A5 11"</t>
+  </si>
+  <si>
+    <t>kf_416a5_12.5i_barrel</t>
+  </si>
+  <si>
+    <t>KF416A5 12.5"</t>
+  </si>
+  <si>
+    <t>kf_416d_14.5i_barrel</t>
+  </si>
+  <si>
+    <t>KF416D 14.5"</t>
+  </si>
+  <si>
+    <t>kf_416a5_14.5i_barrel</t>
+  </si>
+  <si>
+    <t>KF416A5 14.5"</t>
+  </si>
+  <si>
+    <t>kf_416d_16.5i_barrel</t>
+  </si>
+  <si>
+    <t>KF416D 16.5"</t>
+  </si>
+  <si>
+    <t>kf_416a5_16.5i_barrel</t>
+  </si>
+  <si>
+    <t>KF416A5 16.5"</t>
+  </si>
+  <si>
+    <t>kf_416d_20i_barrel</t>
+  </si>
+  <si>
+    <t>KF416D 20"</t>
+  </si>
+  <si>
+    <t>kf_416a5_20i_barrel</t>
+  </si>
+  <si>
+    <t>KF416A5 20"</t>
+  </si>
+  <si>
+    <t>steyr_aug_hbar_620mm_heavy_barrel</t>
+  </si>
+  <si>
+    <t>Löwenhurz 24.4in AUG HBAR</t>
+  </si>
+  <si>
+    <t>steyr_aug_508mm_barrel</t>
+  </si>
+  <si>
+    <t>Löwenherz AUG A3 5.56x45 508mm</t>
+  </si>
+  <si>
+    <t>steyr_aug_457mm_barrel</t>
+  </si>
+  <si>
+    <t>Löwenherz AUG A3 5.56x45 457mm</t>
   </si>
   <si>
     <t>steyr_aug_407mm_barrel</t>
   </si>
   <si>
-    <t>Steyr AUG A3 5.56x45 407mm</t>
-  </si>
-  <si>
-    <t>steyr_aug_508mm_barrel</t>
-  </si>
-  <si>
-    <t>Steyr AUG A3 5.56x45 508mm</t>
+    <t>Löwenherz AUG A3 5.56x45 407mm</t>
   </si>
   <si>
     <t>steyr_aug_350mm_barrel</t>
   </si>
   <si>
-    <t>Steyr AUG A3 5.56x45 350mm</t>
-  </si>
-  <si>
-    <t>steyr_aug_hbar_620mm_heavy_barrel</t>
-  </si>
-  <si>
-    <t>Steyr AUG HBAR 5.56x45 620mm Heavy LMG</t>
-  </si>
-  <si>
-    <t>steyr_aug_457mm_barrel</t>
-  </si>
-  <si>
-    <t>Steyr AUG A3 5.56x45 457mm</t>
-  </si>
-  <si>
-    <t>barrel_deviation</t>
-  </si>
-  <si>
-    <t>buck_barrel_deviation</t>
-  </si>
-  <si>
-    <t>kf_416c_9.0i_barrel</t>
-  </si>
-  <si>
-    <t>KF416C 9.0"</t>
-  </si>
-  <si>
-    <t>kf_416d_10.4i_barrel</t>
-  </si>
-  <si>
-    <t>KF416D 10.4"</t>
-  </si>
-  <si>
-    <t>kf_416a5_11i_barrel</t>
-  </si>
-  <si>
-    <t>KF416A5 11"</t>
-  </si>
-  <si>
-    <t>kf_416a5_12.5i_barrel</t>
-  </si>
-  <si>
-    <t>KF416A5 12.5"</t>
-  </si>
-  <si>
-    <t>kf_416d_14.5i_barrel</t>
-  </si>
-  <si>
-    <t>KF416D 14.5"</t>
-  </si>
-  <si>
-    <t>kf_416a5_14.5i_barrel</t>
-  </si>
-  <si>
-    <t>KF416A5 14.5"</t>
-  </si>
-  <si>
-    <t>kf_416d_16.5i_barrel</t>
-  </si>
-  <si>
-    <t>KF416D 16.5"</t>
-  </si>
-  <si>
-    <t>kf_416a5_16.5i_barrel</t>
-  </si>
-  <si>
-    <t>KF416A5 16.5"</t>
-  </si>
-  <si>
-    <t>kf_416d_20i_barrel</t>
-  </si>
-  <si>
-    <t>KF416D 20"</t>
-  </si>
-  <si>
-    <t>kf_416a5_20i_barrel</t>
-  </si>
-  <si>
-    <t>KF416A5 20"</t>
-  </si>
-  <si>
-    <t>gas</t>
-  </si>
-  <si>
-    <t>whtnls_a1_m4a1_5.56x45_508mm_govt_r_barrel</t>
-  </si>
-  <si>
-    <t>whtnls_m4a1_5.56x45_508mm_hbar_r_barrel</t>
-  </si>
-  <si>
-    <t>ex_call_ar_15_.223wylde_457mm_spiral_6groove_m_barrel</t>
-  </si>
-  <si>
-    <t>whtnls_m4a1_5.56x45_406mm_govt_m_barrel</t>
-  </si>
-  <si>
-    <t>whtnls_m4a1_5.56x45_406mm_socom_c_barrel</t>
-  </si>
-  <si>
-    <t>hart_m4a1_5.56x45_368mm_socom_c_barrel</t>
-  </si>
-  <si>
-    <t>Hart Socom 14.5" Carbine Length Gastube 5.56x45</t>
-  </si>
-  <si>
-    <t>hart_m4a1_5.56x45_368mm_govt_c_barrel</t>
-  </si>
-  <si>
-    <t>Hart Government 14.5" Carbine Length Gastube 5.56x45</t>
-  </si>
-  <si>
-    <t>pac_ks1_5.56x45_348mm_heavy_dimpled_m_barrel</t>
-  </si>
-  <si>
-    <t>hart_m4a1_5.56x45_317mm_govt_c_barrel</t>
-  </si>
-  <si>
-    <t>Hart Government 12.5" Carbine Length Gastube 5.56x45</t>
-  </si>
-  <si>
-    <t>primabarrels_ar15_modern_series_5.56x45_292mm_govt_c_barrel</t>
-  </si>
-  <si>
-    <t>hart_m4a1_5.56x45_267mm_govt_c_barrel</t>
-  </si>
-  <si>
-    <t>Hart Government 10.5" Carbine Length Gastube 5.56x45</t>
-  </si>
-  <si>
-    <t>hart_m4a1_5.56x45_190mm_govt_p_barrel</t>
-  </si>
-  <si>
-    <t>Hart Government 7.5" Pistol Length Gastube 5.56x45</t>
-  </si>
-  <si>
-    <t>quix_tacticals_ar15_127mm_5.56_nitride_barrel_custom_gastube</t>
-  </si>
-  <si>
-    <t>dev</t>
-  </si>
-  <si>
-    <t>old weight</t>
-  </si>
-  <si>
-    <t>new weight</t>
+    <t>Löwenherz AUG A3 5.56x45 350mm</t>
   </si>
   <si>
     <t>aft_mk_16_457mm_barrel</t>
   </si>
   <si>
+    <t>AFT MK-16 457mm</t>
+  </si>
+  <si>
     <t>aft_mk_16_355mm_barrel</t>
   </si>
   <si>
+    <t>AFT MK-16 355mm</t>
+  </si>
+  <si>
     <t>aft_mk_16_254mm_barrel</t>
+  </si>
+  <si>
+    <t>AFT MK-16 254mm</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri Light"/>
-      <family val="2"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C5700"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -449,188 +322,15 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -638,205 +338,16 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="42">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1169,22 +680,22 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>6</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>7</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>8</v>
-      </c>
-      <c r="H2" t="s">
-        <v>42</v>
       </c>
       <c r="I2" t="s">
         <v>9</v>
@@ -1193,48 +704,48 @@
         <v>10</v>
       </c>
       <c r="K2" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="L2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N2" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="P2" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="Q2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="R2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S2" t="s">
-        <v>84</v>
+        <v>18</v>
       </c>
       <c r="T2" t="s">
-        <v>64</v>
+        <v>19</v>
       </c>
       <c r="U2" t="s">
-        <v>85</v>
+        <v>20</v>
       </c>
       <c r="V2" t="s">
-        <v>83</v>
+        <v>21</v>
       </c>
       <c r="X2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C3">
         <v>-12</v>
@@ -1264,7 +775,7 @@
         <v>5000</v>
       </c>
       <c r="N3">
-        <f>C3-D3*20-E3*0.8-F3*0.6-H3*5+I3*15+J3/300</f>
+        <f t="shared" ref="N3:N39" si="0">C3-D3*20-E3*0.8-F3*0.6-H3*5+I3*15+J3/300</f>
         <v>-2.0266666666666655</v>
       </c>
       <c r="P3">
@@ -1277,34 +788,34 @@
         <v>0</v>
       </c>
       <c r="S3">
-        <f>ROUND(Q3*0.035+P3+R3, 2)</f>
+        <f t="shared" ref="S3:S17" si="1">ROUND(Q3*0.035+P3+R3, 2)</f>
         <v>1.02</v>
       </c>
       <c r="T3" s="1">
         <v>0.04</v>
       </c>
       <c r="U3">
-        <f>0.06+0.037*Q3+T3+R3</f>
+        <f t="shared" ref="U3:U38" si="2">0.06+0.037*Q3+T3+R3</f>
         <v>0.98799999999999999</v>
       </c>
       <c r="V3">
-        <f>0+(Q3-14.5)*-0.043</f>
+        <f t="shared" ref="V3:V38" si="3">0+(Q3-14.5)*-0.043</f>
         <v>-0.40849999999999997</v>
       </c>
       <c r="X3">
         <v>349.95</v>
       </c>
       <c r="Y3">
-        <f>X3*6</f>
+        <f t="shared" ref="Y3:Y10" si="4">X3*6</f>
         <v>2099.6999999999998</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="C4">
         <v>-9</v>
@@ -1334,7 +845,7 @@
         <v>1600</v>
       </c>
       <c r="N4">
-        <f t="shared" ref="N4:N39" si="0">C4-D4*20-E4*0.8-F4*0.6-H4*5+I4*15+J4/300</f>
+        <f t="shared" si="0"/>
         <v>-6.8533333333333344</v>
       </c>
       <c r="P4">
@@ -1344,25 +855,25 @@
         <v>20</v>
       </c>
       <c r="S4">
-        <f t="shared" ref="S4:S17" si="1">ROUND(Q4*0.035+P4+R4, 2)</f>
+        <f t="shared" si="1"/>
         <v>0.88</v>
       </c>
       <c r="T4">
         <v>0.04</v>
       </c>
       <c r="U4">
-        <f t="shared" ref="U4:U38" si="2">0.06+0.037*Q4+T4+R4</f>
+        <f t="shared" si="2"/>
         <v>0.84000000000000008</v>
       </c>
       <c r="V4">
-        <f t="shared" ref="V4:V38" si="3">0+(Q4-14.5)*-0.043</f>
+        <f t="shared" si="3"/>
         <v>-0.23649999999999999</v>
       </c>
       <c r="X4">
         <v>344.99</v>
       </c>
       <c r="Y4">
-        <f t="shared" ref="Y4:Y17" si="4">X4*6</f>
+        <f t="shared" si="4"/>
         <v>2069.94</v>
       </c>
       <c r="AA4">
@@ -1372,10 +883,10 @@
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="C5">
         <v>-10</v>
@@ -1442,10 +953,10 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>67</v>
+        <v>29</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="C6">
         <v>-7</v>
@@ -1512,10 +1023,10 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>68</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="C7">
         <v>-4</v>
@@ -1579,10 +1090,10 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="C8">
         <v>-3</v>
@@ -1646,10 +1157,10 @@
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="C9">
         <v>-1</v>
@@ -1713,10 +1224,10 @@
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>72</v>
+        <v>37</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>38</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -1774,10 +1285,10 @@
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -1837,10 +1348,10 @@
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>41</v>
       </c>
       <c r="B12" t="s">
-        <v>76</v>
+        <v>42</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -1895,16 +1406,16 @@
         <v>338</v>
       </c>
       <c r="Y12">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="Y12:Y17" si="5">X12*6</f>
         <v>2028</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="C13">
         <v>2</v>
@@ -1959,16 +1470,16 @@
         <v>155</v>
       </c>
       <c r="Y13">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>930</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="B14" t="s">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="C14">
         <v>3</v>
@@ -2023,16 +1534,16 @@
         <v>299</v>
       </c>
       <c r="Y14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1794</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>80</v>
+        <v>47</v>
       </c>
       <c r="B15" t="s">
-        <v>81</v>
+        <v>48</v>
       </c>
       <c r="C15">
         <v>4</v>
@@ -2087,16 +1598,16 @@
         <v>0.30099999999999999</v>
       </c>
       <c r="Y15">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>82</v>
+        <v>49</v>
       </c>
       <c r="B16" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="C16">
         <v>5</v>
@@ -2154,16 +1665,16 @@
         <v>149.94999999999999</v>
       </c>
       <c r="Y16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>899.69999999999993</v>
       </c>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="C17">
         <v>6</v>
@@ -2221,7 +1732,7 @@
         <v>0.53749999999999998</v>
       </c>
       <c r="Y17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -2241,10 +1752,10 @@
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="B19" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="C19">
         <v>4</v>
@@ -2298,10 +1809,10 @@
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="B20" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="C20">
         <v>3</v>
@@ -2341,7 +1852,7 @@
         <v>0.02</v>
       </c>
       <c r="S20">
-        <f t="shared" ref="S20:S28" si="5">ROUND(Q20*0.033+P49+R20, 2)</f>
+        <f t="shared" ref="S20:S28" si="6">ROUND(Q20*0.033+P49+R20, 2)</f>
         <v>0.36</v>
       </c>
       <c r="U20">
@@ -2355,10 +1866,10 @@
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="C21">
         <v>2</v>
@@ -2398,7 +1909,7 @@
         <v>0</v>
       </c>
       <c r="S21">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.36</v>
       </c>
       <c r="U21">
@@ -2412,10 +1923,10 @@
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="B22" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -2455,7 +1966,7 @@
         <v>0</v>
       </c>
       <c r="S22">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.41</v>
       </c>
       <c r="U22">
@@ -2469,10 +1980,10 @@
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="B23" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -2512,7 +2023,7 @@
         <v>0.05</v>
       </c>
       <c r="S23">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.53</v>
       </c>
       <c r="U23">
@@ -2526,10 +2037,10 @@
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -2569,7 +2080,7 @@
         <v>0.02</v>
       </c>
       <c r="S24">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.5</v>
       </c>
       <c r="U24">
@@ -2583,10 +2094,10 @@
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B25" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="C25">
         <v>-3</v>
@@ -2626,7 +2137,7 @@
         <v>0.05</v>
       </c>
       <c r="S25">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.59</v>
       </c>
       <c r="U25">
@@ -2640,10 +2151,10 @@
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C26">
         <v>-3</v>
@@ -2683,7 +2194,7 @@
         <v>0.02</v>
       </c>
       <c r="S26">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.56000000000000005</v>
       </c>
       <c r="U26">
@@ -2697,10 +2208,10 @@
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="B27" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C27">
         <v>-7</v>
@@ -2740,7 +2251,7 @@
         <v>0.05</v>
       </c>
       <c r="S27">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.71</v>
       </c>
       <c r="U27">
@@ -2754,10 +2265,10 @@
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="B28" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="C28">
         <v>-7</v>
@@ -2797,7 +2308,7 @@
         <v>0.02</v>
       </c>
       <c r="S28">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.68</v>
       </c>
       <c r="U28">
@@ -2828,11 +2339,11 @@
         <v>0</v>
       </c>
       <c r="S29">
-        <f t="shared" ref="S29:S34" si="6">ROUND(Q29*0.033+P29+R29, 2)</f>
+        <f t="shared" ref="S29:S39" si="7">ROUND(Q29*0.033+P29+R29, 2)</f>
         <v>0</v>
       </c>
       <c r="U29">
-        <f t="shared" ref="U29:U34" si="7">0.06+0.037*Q29+T29+R29</f>
+        <f t="shared" si="2"/>
         <v>0.06</v>
       </c>
       <c r="V29">
@@ -2842,26 +2353,26 @@
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>39</v>
+        <v>74</v>
       </c>
       <c r="C30" s="1">
         <v>-10</v>
       </c>
       <c r="D30" s="1">
-        <v>1.01</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="E30" s="1">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="F30" s="1">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="G30" s="1"/>
       <c r="H30" s="1">
-        <v>0.1</v>
+        <v>-0.12</v>
       </c>
       <c r="I30" s="1">
         <v>0.21</v>
@@ -2876,7 +2387,7 @@
       </c>
       <c r="N30">
         <f t="shared" si="0"/>
-        <v>-15.453333333333331</v>
+        <v>-15.753333333333336</v>
       </c>
       <c r="P30">
         <v>0.1</v>
@@ -2888,11 +2399,11 @@
         <v>0.1</v>
       </c>
       <c r="S30">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1.01</v>
       </c>
       <c r="U30">
-        <f t="shared" si="7"/>
+        <f t="shared" si="2"/>
         <v>1.0631478000000001</v>
       </c>
       <c r="V30">
@@ -2902,10 +2413,10 @@
     </row>
     <row r="31" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="C31" s="1">
         <v>-4</v>
@@ -2945,11 +2456,11 @@
         <v>20</v>
       </c>
       <c r="S31">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.76</v>
       </c>
       <c r="U31">
-        <f t="shared" si="7"/>
+        <f t="shared" si="2"/>
         <v>0.8</v>
       </c>
       <c r="V31">
@@ -2959,10 +2470,10 @@
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>40</v>
+        <v>77</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="C32" s="1">
         <v>-2</v>
@@ -3002,11 +2513,11 @@
         <v>17.992100000000001</v>
       </c>
       <c r="S32">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.69</v>
       </c>
       <c r="U32">
-        <f t="shared" si="7"/>
+        <f t="shared" si="2"/>
         <v>0.72570770000000007</v>
       </c>
       <c r="V32">
@@ -3016,10 +2527,10 @@
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>33</v>
+        <v>80</v>
       </c>
       <c r="C33" s="1">
         <v>0</v>
@@ -3059,11 +2570,11 @@
         <v>16.023599999999998</v>
       </c>
       <c r="S33">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.63</v>
       </c>
       <c r="U33">
-        <f t="shared" si="7"/>
+        <f t="shared" si="2"/>
         <v>0.65287319999999993</v>
       </c>
       <c r="V33">
@@ -3073,10 +2584,10 @@
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>36</v>
+        <v>81</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>37</v>
+        <v>82</v>
       </c>
       <c r="C34" s="1">
         <v>2</v>
@@ -3116,11 +2627,11 @@
         <v>13.779500000000001</v>
       </c>
       <c r="S34">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.55000000000000004</v>
       </c>
       <c r="U34">
-        <f t="shared" si="7"/>
+        <f t="shared" si="2"/>
         <v>0.56984149999999989</v>
       </c>
       <c r="V34">
@@ -3147,7 +2658,7 @@
         <v>0</v>
       </c>
       <c r="S35">
-        <f t="shared" ref="S35:S39" si="8">ROUND(Q35*0.033+P35+R35, 2)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="U35">
@@ -3161,10 +2672,10 @@
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>31</v>
+        <v>84</v>
       </c>
       <c r="C36" s="1">
         <v>-5</v>
@@ -3204,7 +2715,7 @@
         <v>17.992100000000001</v>
       </c>
       <c r="S36">
-        <f>ROUND(Q36*0.033+P36+R36, 2)</f>
+        <f t="shared" si="7"/>
         <v>0.73</v>
       </c>
       <c r="U36">
@@ -3218,10 +2729,10 @@
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>30</v>
+        <v>86</v>
       </c>
       <c r="C37" s="1">
         <v>0</v>
@@ -3261,7 +2772,7 @@
         <v>13.9764</v>
       </c>
       <c r="S37">
-        <f>ROUND(Q37*0.033+P37+R37, 2)</f>
+        <f t="shared" si="7"/>
         <v>0.6</v>
       </c>
       <c r="U37">
@@ -3275,10 +2786,10 @@
     </row>
     <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>29</v>
       </c>
       <c r="C38" s="1">
         <v>2</v>
@@ -3318,7 +2829,7 @@
         <v>10</v>
       </c>
       <c r="S38">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>0.47</v>
       </c>
       <c r="U38">
@@ -3349,7 +2860,7 @@
         <v>0</v>
       </c>
       <c r="S39">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -3460,6 +2971,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update aug hbar barrel name again
</commit_message>
<xml_diff>
--- a/changes/556-barrels.xlsx
+++ b/changes/556-barrels.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yifan/Documents/deadline-balancing/changes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ACB0132-3513-8547-BAEA-F7D8B1667938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37B2CFD3-7CAC-40B9-AF4C-21049F1CC3E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="m4-barrels" sheetId="1" r:id="rId1"/>
@@ -254,9 +254,6 @@
     <t>KF416A5 20"</t>
   </si>
   <si>
-    <t>Löwenhurz AUG HBAR 24.4"</t>
-  </si>
-  <si>
     <t>steyr_aug_508mm_barrel</t>
   </si>
   <si>
@@ -300,6 +297,9 @@
   </si>
   <si>
     <t>lowenhurz_aug_hbar_620mm_heavy_barrel</t>
+  </si>
+  <si>
+    <t>Löwenhurz AUG HBAR 620mm</t>
   </si>
 </sst>
 </file>
@@ -660,19 +660,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.5" customWidth="1"/>
-    <col min="2" max="2" width="27.1640625" customWidth="1"/>
-    <col min="3" max="25" width="6.6640625" customWidth="1"/>
+    <col min="1" max="1" width="29.42578125" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" customWidth="1"/>
+    <col min="3" max="25" width="6.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -740,7 +740,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -810,7 +810,7 @@
         <v>2099.6999999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -881,7 +881,7 @@
         <v>0.80681818181818177</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -951,7 +951,7 @@
         <v>2099.94</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -1021,7 +1021,7 @@
         <v>2232</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>31</v>
       </c>
@@ -1088,7 +1088,7 @@
         <v>1979.94</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -1155,7 +1155,7 @@
         <v>1679.94</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -1222,7 +1222,7 @@
         <v>2094</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>37</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>39</v>
       </c>
@@ -1346,7 +1346,7 @@
         <v>3.4400000000000028E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>41</v>
       </c>
@@ -1410,7 +1410,7 @@
         <v>2028</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -1474,7 +1474,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>45</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>1794</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>47</v>
       </c>
@@ -1602,7 +1602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>49</v>
       </c>
@@ -1669,7 +1669,7 @@
         <v>899.69999999999993</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>51</v>
       </c>
@@ -1736,7 +1736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="N18">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1750,7 +1750,7 @@
         <v>0.62349999999999994</v>
       </c>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>53</v>
       </c>
@@ -1807,7 +1807,7 @@
         <v>0.23649999999999999</v>
       </c>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>55</v>
       </c>
@@ -1864,7 +1864,7 @@
         <v>0.17629999999999996</v>
       </c>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>57</v>
       </c>
@@ -1921,7 +1921,7 @@
         <v>0.15049999999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>59</v>
       </c>
@@ -1978,7 +1978,7 @@
         <v>8.5999999999999993E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>61</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>63</v>
       </c>
@@ -2092,7 +2092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>65</v>
       </c>
@@ -2149,7 +2149,7 @@
         <v>-8.5999999999999993E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>67</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>-8.5999999999999993E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>69</v>
       </c>
@@ -2263,7 +2263,7 @@
         <v>-0.23649999999999999</v>
       </c>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>71</v>
       </c>
@@ -2320,7 +2320,7 @@
         <v>-0.23649999999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -2351,12 +2351,12 @@
         <v>0.62349999999999994</v>
       </c>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="C30" s="1">
         <v>-8</v>
@@ -2411,12 +2411,12 @@
         <v>-0.42610420000000004</v>
       </c>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="C31" s="1">
         <v>-4</v>
@@ -2468,12 +2468,12 @@
         <v>-0.23649999999999999</v>
       </c>
     </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="C32" s="1">
         <v>-2</v>
@@ -2525,12 +2525,12 @@
         <v>-0.15016030000000002</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>79</v>
       </c>
       <c r="C33" s="1">
         <v>0</v>
@@ -2582,12 +2582,12 @@
         <v>-6.5514799999999915E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>81</v>
       </c>
       <c r="C34" s="1">
         <v>2</v>
@@ -2639,7 +2639,7 @@
         <v>3.0981499999999974E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -2670,12 +2670,12 @@
         <v>0.62349999999999994</v>
       </c>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="C36" s="1">
         <v>-5</v>
@@ -2727,12 +2727,12 @@
         <v>-0.15016030000000002</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>85</v>
       </c>
       <c r="C37" s="1">
         <v>0</v>
@@ -2784,12 +2784,12 @@
         <v>2.2514800000000001E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>87</v>
       </c>
       <c r="C38" s="1">
         <v>2</v>
@@ -2841,7 +2841,7 @@
         <v>0.19349999999999998</v>
       </c>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -2864,7 +2864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -2879,7 +2879,7 @@
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -2894,7 +2894,7 @@
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -2909,7 +2909,7 @@
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -2924,7 +2924,7 @@
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -2939,7 +2939,7 @@
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -2954,7 +2954,7 @@
       <c r="L45" s="1"/>
       <c r="M45" s="1"/>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>

</xml_diff>